<commit_message>
Improve portal UI, Mermaid support, and wallpaper management
- Add Mermaid rendering for blog and wiki markdown
- Introduce wallpaper manifest and slug-based video naming
- Refresh wiki/browse templates and mp-portal styling
- Add event image uploads and update site data spreadsheet

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/zhita_settings.xlsx
+++ b/zhita_settings.xlsx
@@ -4727,7 +4727,6 @@
       <c r="C27" t="n">
         <v>30</v>
       </c>
-      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
           <t>整体情绪呈现从深度焦虑和虚无向逐步接纳、反思与温和希望过渡的U型趋势。</t>
@@ -4757,7 +4756,6 @@
       <c r="C28" t="n">
         <v>30</v>
       </c>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
           <t>整体情绪呈现从深度焦虑和虚无向波动性接纳与成长转变的趋势，在自我怀疑与深刻反思中螺旋式上升。</t>
@@ -4787,7 +4785,6 @@
       <c r="C29" t="n">
         <v>30</v>
       </c>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
           <t>整体情绪呈现从深度焦虑、虚无向阶段性接纳与微弱成长过渡的“U型”波动趋势，但根基仍不稳定。</t>
@@ -4838,7 +4835,6 @@
           <t>3月的狮子</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -4846,7 +4842,6 @@
           <t>AIR</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -4854,7 +4849,6 @@
           <t>Angles of Death</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -4994,7 +4988,6 @@
           <t>Just Because!</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -5122,7 +5115,6 @@
           <t>一个人的○○小日子</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -5154,7 +5146,6 @@
           <t>一起一起这里那里</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -5162,7 +5153,6 @@
           <t>三体</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -5170,7 +5160,6 @@
           <t>三坪房间的侵略者！</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -5178,7 +5167,6 @@
           <t>不动声色的柏田与喜形于色的太田</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -5186,7 +5174,6 @@
           <t>不知情的转学生硬要凑上来</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -5194,7 +5181,6 @@
           <t>世界顶尖的暗杀者，转生为异世界贵族</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -5226,7 +5212,6 @@
           <t>久保同学不放过我</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -5258,7 +5243,6 @@
           <t>人间失格</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -5326,7 +5310,6 @@
           <t>会长是女仆大人！</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -5334,7 +5317,6 @@
           <t>伪恋</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -5342,7 +5324,6 @@
           <t>你与我最后的战场，亦或是世界起始的圣战</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -5350,7 +5331,6 @@
           <t>侦探已死</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -5358,7 +5338,6 @@
           <t>俺物语</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -5402,7 +5381,6 @@
           <t>全员恶玉</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -5410,7 +5388,6 @@
           <t>公司的小小前辈</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -5418,7 +5395,6 @@
           <t>关于前辈很烦人的事</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -5450,7 +5426,6 @@
           <t>冰属性男子和酷酷女同事</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5482,7 +5457,6 @@
           <t>冰菓</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5490,7 +5464,6 @@
           <t>别当欧尼酱了！</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5522,7 +5495,6 @@
           <t>变态王子与不笑猫</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5530,7 +5502,6 @@
           <t>只要贝尔哲布布大小姐喜欢就好</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5538,7 +5509,6 @@
           <t>告白实行委员会</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5582,7 +5552,6 @@
           <t>品酒要在成为夫妻后</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -5590,7 +5559,6 @@
           <t>喜欢本大爷的竟然就你一个？</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -5646,7 +5614,6 @@
           <t>因为是反派大小姐所以养了魔王</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -5654,7 +5621,6 @@
           <t>国王排名</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -5662,7 +5628,6 @@
           <t>在下坂本，有何贵干？</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -5670,7 +5635,6 @@
           <t>在魔王城说晚安</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -5702,7 +5666,6 @@
           <t>坂本日常</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -5710,7 +5673,6 @@
           <t>埃罗芒阿老师</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -5718,7 +5680,6 @@
           <t>城下町的蒲公英</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -5726,7 +5687,6 @@
           <t>堀与宫村</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -5746,7 +5706,6 @@
           <t>夏日口袋</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -5754,7 +5713,6 @@
           <t>夏日幻魂</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -5762,7 +5720,6 @@
           <t>夏日重现</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -5794,7 +5751,6 @@
           <t>多田君不恋爱</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -5802,7 +5758,6 @@
           <t>大叔与棉花糖</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -5810,7 +5765,6 @@
           <t>大正少女御伽话</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -5818,7 +5772,6 @@
           <t>大理寺日志</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -5826,7 +5779,6 @@
           <t>天使降临到我身边</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -5834,7 +5786,6 @@
           <t>奇幻世界舅舅</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -5842,7 +5793,6 @@
           <t>女孩的钓鱼慢活</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -5850,7 +5800,6 @@
           <t>如果能写小说就好了</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -5858,7 +5807,6 @@
           <t>孤独摇滚</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -5890,7 +5838,6 @@
           <t>宝石之国</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -5910,7 +5857,6 @@
           <t>小桃小栗 Love Love物语</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -5918,7 +5864,6 @@
           <t>小森同学拒绝不了！</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -5926,7 +5871,6 @@
           <t>少女终末旅行</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -5934,7 +5878,6 @@
           <t>尽管如此世界依然美丽</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -5942,7 +5885,6 @@
           <t>川柳少女</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -5998,7 +5940,6 @@
           <t>异度入侵</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -6006,7 +5947,6 @@
           <t>式守同学不只可爱而已</t>
         </is>
       </c>
-      <c r="B118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -6038,7 +5978,6 @@
           <t>徒然喜欢你</t>
         </is>
       </c>
-      <c r="B121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -6046,7 +5985,6 @@
           <t>心灵想要大声呼喊</t>
         </is>
       </c>
-      <c r="B122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -6102,7 +6040,6 @@
           <t>恋旅</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr"/>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -6110,7 +6047,6 @@
           <t>恶魔奶爸</t>
         </is>
       </c>
-      <c r="B128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -6118,7 +6054,6 @@
           <t>我们仍未知道那天所见的花的名字。</t>
         </is>
       </c>
-      <c r="B129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -6126,7 +6061,6 @@
           <t>我们大家的河合庄</t>
         </is>
       </c>
-      <c r="B130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -6134,7 +6068,6 @@
           <t>我们无法一起学习</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -6142,7 +6075,6 @@
           <t>我女友与青梅竹马的惨烈修罗场</t>
         </is>
       </c>
-      <c r="B132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -6234,7 +6166,6 @@
           <t>我被逐出队伍后过上慢生活</t>
         </is>
       </c>
-      <c r="B140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -6242,7 +6173,6 @@
           <t>我，不是说了能力要平均值么！</t>
         </is>
       </c>
-      <c r="B141" t="inlineStr"/>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -6250,7 +6180,6 @@
           <t>房东青春期！</t>
         </is>
       </c>
-      <c r="B142" t="inlineStr"/>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -6306,7 +6235,6 @@
           <t>捡到退婚大小姐的我，教她幸福的事</t>
         </is>
       </c>
-      <c r="B147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -6362,7 +6290,6 @@
           <t>散华礼弥</t>
         </is>
       </c>
-      <c r="B152" t="inlineStr"/>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -6370,7 +6297,6 @@
           <t>敦君与女朋友</t>
         </is>
       </c>
-      <c r="B153" t="inlineStr"/>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -6438,7 +6364,6 @@
           <t>无能力者娜娜</t>
         </is>
       </c>
-      <c r="B159" t="inlineStr"/>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -6446,7 +6371,6 @@
           <t>日常</t>
         </is>
       </c>
-      <c r="B160" t="inlineStr"/>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -6454,7 +6378,6 @@
           <t>明日酱的水手服</t>
         </is>
       </c>
-      <c r="B161" t="inlineStr"/>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -6462,7 +6385,6 @@
           <t>暂停！让我查攻略</t>
         </is>
       </c>
-      <c r="B162" t="inlineStr"/>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -6494,7 +6416,6 @@
           <t>月刊少女野崎君</t>
         </is>
       </c>
-      <c r="B165" t="inlineStr"/>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -6502,7 +6423,6 @@
           <t>月色真美</t>
         </is>
       </c>
-      <c r="B166" t="inlineStr"/>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -6510,7 +6430,6 @@
           <t>未确认进行式</t>
         </is>
       </c>
-      <c r="B167" t="inlineStr"/>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -6518,7 +6437,6 @@
           <t>极主夫道</t>
         </is>
       </c>
-      <c r="B168" t="inlineStr"/>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -6526,7 +6444,6 @@
           <t>林家的天使同学</t>
         </is>
       </c>
-      <c r="B169" t="inlineStr"/>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -6546,7 +6463,6 @@
           <t>某科学的一方通行</t>
         </is>
       </c>
-      <c r="B171" t="inlineStr"/>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -6590,7 +6506,6 @@
           <t>樱花庄的宠物女孩</t>
         </is>
       </c>
-      <c r="B175" t="inlineStr"/>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -6646,7 +6561,6 @@
           <t>正相反的你与我</t>
         </is>
       </c>
-      <c r="B180" t="inlineStr"/>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -6654,7 +6568,6 @@
           <t>武装少女</t>
         </is>
       </c>
-      <c r="B181" t="inlineStr"/>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -6662,7 +6575,6 @@
           <t>死神少爷与黑女仆</t>
         </is>
       </c>
-      <c r="B182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -6730,7 +6642,6 @@
           <t>温暖的印记</t>
         </is>
       </c>
-      <c r="B188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -6738,7 +6649,6 @@
           <t>游戏人生</t>
         </is>
       </c>
-      <c r="B189" t="inlineStr"/>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -6746,7 +6656,6 @@
           <t>漂流少年</t>
         </is>
       </c>
-      <c r="B190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -6754,7 +6663,6 @@
           <t>熏香花朵凛然绽放</t>
         </is>
       </c>
-      <c r="B191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -6762,7 +6670,6 @@
           <t>爱幽的密室</t>
         </is>
       </c>
-      <c r="B192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -6770,7 +6677,6 @@
           <t>狼少女与黑王子</t>
         </is>
       </c>
-      <c r="B193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -6778,7 +6684,6 @@
           <t>玉子市场</t>
         </is>
       </c>
-      <c r="B194" t="inlineStr"/>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -6786,7 +6691,6 @@
           <t>玉子的爱情故事</t>
         </is>
       </c>
-      <c r="B195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -6818,7 +6722,6 @@
           <t>理科生坠入情网，故尝试证明。</t>
         </is>
       </c>
-      <c r="B198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -6826,7 +6729,6 @@
           <t>瓦尼塔斯的手记</t>
         </is>
       </c>
-      <c r="B199" t="inlineStr"/>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -6834,7 +6736,6 @@
           <t>甘城光辉游乐园</t>
         </is>
       </c>
-      <c r="B200" t="inlineStr"/>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -6842,7 +6743,6 @@
           <t>田中君总是如此慵懒</t>
         </is>
       </c>
-      <c r="B201" t="inlineStr"/>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -6874,7 +6774,6 @@
           <t>白圣女与黑牧师</t>
         </is>
       </c>
-      <c r="B204" t="inlineStr"/>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -6882,7 +6781,6 @@
           <t>百变的七仓同学</t>
         </is>
       </c>
-      <c r="B205" t="inlineStr"/>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -6890,7 +6788,6 @@
           <t>真理面具</t>
         </is>
       </c>
-      <c r="B206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -6898,7 +6795,6 @@
           <t>知晓天空之蓝的人啊</t>
         </is>
       </c>
-      <c r="B207" t="inlineStr"/>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -6930,7 +6826,6 @@
           <t>端脑</t>
         </is>
       </c>
-      <c r="B210" t="inlineStr"/>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -6938,7 +6833,6 @@
           <t>笨女孩</t>
         </is>
       </c>
-      <c r="B211" t="inlineStr"/>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -7018,7 +6912,6 @@
           <t>线上游戏的队友不可能是女生？</t>
         </is>
       </c>
-      <c r="B218" t="inlineStr"/>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -7026,7 +6919,6 @@
           <t>终物语</t>
         </is>
       </c>
-      <c r="B219" t="inlineStr"/>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -7034,7 +6926,6 @@
           <t>继母的拖油瓶是我前女友</t>
         </is>
       </c>
-      <c r="B220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -7042,7 +6933,6 @@
           <t>老夫老妻重返青春</t>
         </is>
       </c>
-      <c r="B221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -7098,7 +6988,6 @@
           <t>花开伊吕波</t>
         </is>
       </c>
-      <c r="B226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -7106,7 +6995,6 @@
           <t>花果山传</t>
         </is>
       </c>
-      <c r="B227" t="inlineStr"/>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -7114,7 +7002,6 @@
           <t>莉可丽丝</t>
         </is>
       </c>
-      <c r="B228" t="inlineStr"/>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -7122,7 +7009,6 @@
           <t>萤火之森</t>
         </is>
       </c>
-      <c r="B229" t="inlineStr"/>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -7154,7 +7040,6 @@
           <t>虚构推理</t>
         </is>
       </c>
-      <c r="B232" t="inlineStr"/>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -7162,7 +7047,6 @@
           <t>虫师</t>
         </is>
       </c>
-      <c r="B233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -7170,7 +7054,6 @@
           <t>被神捡到的男人</t>
         </is>
       </c>
-      <c r="B234" t="inlineStr"/>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -7178,7 +7061,6 @@
           <t>见面5秒开始战斗</t>
         </is>
       </c>
-      <c r="B235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -7186,7 +7068,6 @@
           <t>言叶之庭</t>
         </is>
       </c>
-      <c r="B236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -7242,7 +7123,6 @@
           <t>超人高中生们即便在异世界也能从容生存！</t>
         </is>
       </c>
-      <c r="B241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -7250,7 +7130,6 @@
           <t>跃动青春</t>
         </is>
       </c>
-      <c r="B242" t="inlineStr"/>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
@@ -7474,7 +7353,6 @@
           <t>这个美术社大有问题！</t>
         </is>
       </c>
-      <c r="B261" t="inlineStr"/>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
@@ -7482,7 +7360,6 @@
           <t>迷宫饭</t>
         </is>
       </c>
-      <c r="B262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -7490,7 +7367,6 @@
           <t>邻桌的怪同学</t>
         </is>
       </c>
-      <c r="B263" t="inlineStr"/>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
@@ -7498,7 +7374,6 @@
           <t>酷爱电影的庞波小姐</t>
         </is>
       </c>
-      <c r="B264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -7542,7 +7417,6 @@
           <t>阳光中的青时雨</t>
         </is>
       </c>
-      <c r="B268" t="inlineStr"/>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
@@ -7550,7 +7424,6 @@
           <t>阿宅的恋爱真难</t>
         </is>
       </c>
-      <c r="B269" t="inlineStr"/>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
@@ -7558,7 +7431,6 @@
           <t>雾山五行</t>
         </is>
       </c>
-      <c r="B270" t="inlineStr"/>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
@@ -7566,7 +7438,6 @@
           <t>青春之旅</t>
         </is>
       </c>
-      <c r="B271" t="inlineStr"/>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
@@ -7694,7 +7565,6 @@
           <t>魔法禁书目录</t>
         </is>
       </c>
-      <c r="B282" t="inlineStr"/>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
@@ -7702,7 +7572,6 @@
           <t>龙与虎</t>
         </is>
       </c>
-      <c r="B283" t="inlineStr"/>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -7800,7 +7669,6 @@
           <t>企鹅公路</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -7808,7 +7676,6 @@
           <t>声之形</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -7816,7 +7683,6 @@
           <t>大鱼海棠</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -7824,7 +7690,6 @@
           <t>天气之子</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -7832,7 +7697,6 @@
           <t>姜子牙</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -7840,7 +7704,6 @@
           <t>新神榜：哪吒重生</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -7848,7 +7711,6 @@
           <t>机器人总动员</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -7856,7 +7718,6 @@
           <t>浪浪山小妖怪</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -7864,7 +7725,6 @@
           <t>海兽之子</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -7872,7 +7732,6 @@
           <t>深海</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -7880,7 +7739,6 @@
           <t>烟花</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -7936,7 +7794,6 @@
           <t>白蛇2：青蛇劫起</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -7944,7 +7801,6 @@
           <t>秒速五厘米</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -7952,7 +7808,6 @@
           <t>罗小黑战记</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -7960,7 +7815,6 @@
           <t>罗小黑战记2</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -7968,7 +7822,6 @@
           <t>言语如苏打般涌现</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -7976,7 +7829,6 @@
           <t>通往夏天的隧道</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -7984,7 +7836,6 @@
           <t>间谍过家家 代号：白</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -7992,7 +7843,6 @@
           <t>飞屋环游记</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -8000,7 +7850,6 @@
           <t>一个叫欧维的男人决定去死</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -8008,7 +7857,6 @@
           <t>一直游到海水变蓝</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -8016,7 +7864,6 @@
           <t>上升：我们一起飞上3万米高空</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -8024,7 +7871,6 @@
           <t>与玛格丽特的午后</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -8032,7 +7878,6 @@
           <t>了不起的盖兹比</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -8136,7 +7981,6 @@
           <t>奥本海默</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -8144,7 +7988,6 @@
           <t>少年派的奇幻漂流</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -8152,7 +7995,6 @@
           <t>当幸福来敲门</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -8160,7 +8002,6 @@
           <t>心灵捕手</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -8168,7 +8009,6 @@
           <t>怦然心动</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -8176,7 +8016,6 @@
           <t>情书</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -8184,7 +8023,6 @@
           <t>我是谁</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -8192,7 +8030,6 @@
           <t>摔跤吧！爸爸</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -8236,7 +8073,6 @@
           <t>星际穿越</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -8244,7 +8080,6 @@
           <t>楚门的世界</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -8252,7 +8087,6 @@
           <t>波西米亚狂想曲</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -8260,7 +8094,6 @@
           <t>泰坦尼克号</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -8280,7 +8113,6 @@
           <t>海蒂和爷爷</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -8288,7 +8120,6 @@
           <t>猫鼠游戏</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -8296,7 +8127,6 @@
           <t>白日梦想家</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -8304,7 +8134,6 @@
           <t>神奇动物在哪里</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -8312,7 +8141,6 @@
           <t>神探夏洛克：可恶的新娘</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -8320,7 +8148,6 @@
           <t>绿皮书</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -8328,7 +8155,6 @@
           <t>罗马假日</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -8336,7 +8162,6 @@
           <t>肖申克的救赎</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -8344,7 +8169,6 @@
           <t>让子弹飞</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -8352,7 +8176,6 @@
           <t>超脱</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -8360,7 +8183,6 @@
           <t>遗愿清单</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -8368,7 +8190,6 @@
           <t>钢琴家</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -8376,7 +8197,6 @@
           <t>阿甘正传</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -8384,7 +8204,6 @@
           <t>飞驰人生</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -8392,7 +8211,6 @@
           <t>魂断蓝桥</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -10349,7 +10167,6 @@
           <t>任翔</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10362,7 +10179,6 @@
           <t>何梦妍</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10375,7 +10191,6 @@
           <t>刘成</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10388,7 +10203,6 @@
           <t>刘滢美</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr"/>
       <c r="C15" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10401,7 +10215,6 @@
           <t>刘畅</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr"/>
       <c r="C16" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10414,7 +10227,6 @@
           <t>史书畅</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr"/>
       <c r="C17" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10427,7 +10239,6 @@
           <t>席莫然</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
       <c r="C18" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10440,7 +10251,6 @@
           <t>张佳琦</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10453,7 +10263,6 @@
           <t>张俊凯</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10466,7 +10275,6 @@
           <t>张子凯</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr"/>
       <c r="C21" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10479,7 +10287,6 @@
           <t>张家旭</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr"/>
       <c r="C22" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10492,7 +10299,6 @@
           <t>张梦凯</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10505,7 +10311,6 @@
           <t>张淑涵</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10518,7 +10323,6 @@
           <t>张琳彤</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10531,7 +10335,6 @@
           <t>张畅</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10544,7 +10347,6 @@
           <t>张笑语</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10557,7 +10359,6 @@
           <t>张锦源</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10570,7 +10371,6 @@
           <t>权家静</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr"/>
       <c r="C29" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10583,7 +10383,6 @@
           <t>权怡萱</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10596,7 +10395,6 @@
           <t>李天一</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10609,7 +10407,6 @@
           <t>李家丞</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10622,7 +10419,6 @@
           <t>李悦熙</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10635,7 +10431,6 @@
           <t>李睿倩</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10648,7 +10443,6 @@
           <t>李鑫万</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10661,7 +10455,6 @@
           <t>杨佳瑛</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10674,7 +10467,6 @@
           <t>梁博勋</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10687,7 +10479,6 @@
           <t>梁昕宇</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10700,7 +10491,6 @@
           <t>梁饮涛</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10713,7 +10503,6 @@
           <t>梅荣琛</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10726,7 +10515,6 @@
           <t>毛书鹏</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10739,7 +10527,6 @@
           <t>汤锦钊</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10752,7 +10539,6 @@
           <t>焦昊晖</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10765,7 +10551,6 @@
           <t>王梦湾</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10778,7 +10563,6 @@
           <t>秦毅轩</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10791,7 +10575,6 @@
           <t>苗家乐</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10804,7 +10587,6 @@
           <t>贾源</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10817,7 +10599,6 @@
           <t>赵灿</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10830,7 +10611,6 @@
           <t>郑秀杰</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10843,7 +10623,6 @@
           <t>郭佩琳</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10856,7 +10635,6 @@
           <t>郭林霄</t>
         </is>
       </c>
-      <c r="B51" t="inlineStr"/>
       <c r="C51" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10869,7 +10647,6 @@
           <t>魏羽萱</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10882,7 +10659,6 @@
           <t>黄媛媛</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
           <t>小学同学</t>
@@ -10895,7 +10671,6 @@
           <t>何思源</t>
         </is>
       </c>
-      <c r="B54" t="inlineStr"/>
       <c r="C54" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -10908,7 +10683,6 @@
           <t>刘冰洁</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -10921,7 +10695,6 @@
           <t>刘映泓</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -10934,7 +10707,6 @@
           <t>卢琦</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr"/>
       <c r="C57" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -10947,7 +10719,6 @@
           <t>吴晓露</t>
         </is>
       </c>
-      <c r="B58" t="inlineStr"/>
       <c r="C58" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -10960,7 +10731,6 @@
           <t>孙一然</t>
         </is>
       </c>
-      <c r="B59" t="inlineStr"/>
       <c r="C59" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -10973,7 +10743,6 @@
           <t>孙宴莹</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -10986,7 +10755,6 @@
           <t>席泽润</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -10999,7 +10767,6 @@
           <t>庞耀翔</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11012,7 +10779,6 @@
           <t>康圣哲</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11025,7 +10791,6 @@
           <t>张世豪</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11038,7 +10803,6 @@
           <t>张俊莹</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11051,7 +10815,6 @@
           <t>张冰虹</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr"/>
       <c r="C66" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11064,7 +10827,6 @@
           <t>张子悦</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11077,7 +10839,6 @@
           <t>张家旭</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11090,7 +10851,6 @@
           <t>张旭欣</t>
         </is>
       </c>
-      <c r="B69" t="inlineStr"/>
       <c r="C69" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11103,7 +10863,6 @@
           <t>张易坤</t>
         </is>
       </c>
-      <c r="B70" t="inlineStr"/>
       <c r="C70" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11116,7 +10875,6 @@
           <t>张智庭</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11129,7 +10887,6 @@
           <t>张智瑛</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11142,7 +10899,6 @@
           <t>张梓阳</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11155,7 +10911,6 @@
           <t>张玉涵</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11168,7 +10923,6 @@
           <t>张笑语</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11181,7 +10935,6 @@
           <t>权家森</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11194,7 +10947,6 @@
           <t>权晨烨</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11207,7 +10959,6 @@
           <t>李尚儒</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr"/>
       <c r="C78" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11220,7 +10971,6 @@
           <t>李煜莹</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr"/>
       <c r="C79" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11233,7 +10983,6 @@
           <t>李煜豪</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr"/>
       <c r="C80" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11246,7 +10995,6 @@
           <t>梁越凡</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11259,7 +11007,6 @@
           <t>梅任江南</t>
         </is>
       </c>
-      <c r="B82" t="inlineStr"/>
       <c r="C82" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11272,7 +11019,6 @@
           <t>王少华</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11285,7 +11031,6 @@
           <t>王新换</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11298,7 +11043,6 @@
           <t>王梦瑶</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr"/>
       <c r="C85" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11311,7 +11055,6 @@
           <t>秦嘉欣</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr"/>
       <c r="C86" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11324,7 +11067,6 @@
           <t>秦毅轩</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr"/>
       <c r="C87" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11337,7 +11079,6 @@
           <t>程前</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr"/>
       <c r="C88" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11350,7 +11091,6 @@
           <t>胡家璇</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr"/>
       <c r="C89" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11363,7 +11103,6 @@
           <t>胡鸿斌</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr"/>
       <c r="C90" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11376,7 +11115,6 @@
           <t>苌晓凡</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr"/>
       <c r="C91" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11389,7 +11127,6 @@
           <t>蒋鑫楠</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr"/>
       <c r="C92" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11402,7 +11139,6 @@
           <t>赵元琳</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr"/>
       <c r="C93" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11415,7 +11151,6 @@
           <t>赵冬夏</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr"/>
       <c r="C94" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11428,7 +11163,6 @@
           <t>郑泽明</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr"/>
       <c r="C95" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11441,7 +11175,6 @@
           <t>酒怡凡</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr"/>
       <c r="C96" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11454,7 +11187,6 @@
           <t>陈家悦</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr"/>
       <c r="C97" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11467,7 +11199,6 @@
           <t>韩庆昱</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr"/>
       <c r="C98" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11480,7 +11211,6 @@
           <t>鲁冰雁</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr"/>
       <c r="C99" t="inlineStr">
         <is>
           <t>初中同学</t>
@@ -11493,7 +11223,6 @@
           <t>上官饮钰</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr"/>
       <c r="C100" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11506,7 +11235,6 @@
           <t>刘一卓</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr"/>
       <c r="C101" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11519,7 +11247,6 @@
           <t>刘泽桂</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr"/>
       <c r="C102" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11532,7 +11259,6 @@
           <t>周佳音</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr"/>
       <c r="C103" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11545,7 +11271,6 @@
           <t>周林旭</t>
         </is>
       </c>
-      <c r="B104" t="inlineStr"/>
       <c r="C104" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11558,7 +11283,6 @@
           <t>和梦颖</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr"/>
       <c r="C105" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11571,7 +11295,6 @@
           <t>姚林杉</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr"/>
       <c r="C106" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11584,7 +11307,6 @@
           <t>姜新原</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr"/>
       <c r="C107" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11597,7 +11319,6 @@
           <t>姬国磊</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr"/>
       <c r="C108" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11610,7 +11331,6 @@
           <t>姬翔</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr"/>
       <c r="C109" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11623,7 +11343,6 @@
           <t>孙云浩</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr"/>
       <c r="C110" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11636,7 +11355,6 @@
           <t>宁俊鹏</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr"/>
       <c r="C111" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11649,7 +11367,6 @@
           <t>安思洁</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr"/>
       <c r="C112" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11662,7 +11379,6 @@
           <t>宋宇衡</t>
         </is>
       </c>
-      <c r="B113" t="inlineStr"/>
       <c r="C113" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11675,7 +11391,6 @@
           <t>宋煜邦</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr"/>
       <c r="C114" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11688,7 +11403,6 @@
           <t>尚进亿</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr"/>
       <c r="C115" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11701,7 +11415,6 @@
           <t>张冰洁</t>
         </is>
       </c>
-      <c r="B116" t="inlineStr"/>
       <c r="C116" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11714,7 +11427,6 @@
           <t>张奕扬</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr"/>
       <c r="C117" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11727,7 +11439,6 @@
           <t>张瑞琦</t>
         </is>
       </c>
-      <c r="B118" t="inlineStr"/>
       <c r="C118" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11740,7 +11451,6 @@
           <t>张静怡</t>
         </is>
       </c>
-      <c r="B119" t="inlineStr"/>
       <c r="C119" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11753,7 +11463,6 @@
           <t>徐丹颖</t>
         </is>
       </c>
-      <c r="B120" t="inlineStr"/>
       <c r="C120" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11766,7 +11475,6 @@
           <t>李广钰</t>
         </is>
       </c>
-      <c r="B121" t="inlineStr"/>
       <c r="C121" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11779,7 +11487,6 @@
           <t>杨思涵</t>
         </is>
       </c>
-      <c r="B122" t="inlineStr"/>
       <c r="C122" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11792,7 +11499,6 @@
           <t>杨思源</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr"/>
       <c r="C123" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11805,7 +11511,6 @@
           <t>杨艳琼</t>
         </is>
       </c>
-      <c r="B124" t="inlineStr"/>
       <c r="C124" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11818,7 +11523,6 @@
           <t>江子航</t>
         </is>
       </c>
-      <c r="B125" t="inlineStr"/>
       <c r="C125" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11831,7 +11535,6 @@
           <t>潘梦歌</t>
         </is>
       </c>
-      <c r="B126" t="inlineStr"/>
       <c r="C126" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11844,7 +11547,6 @@
           <t>牛玉成</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr"/>
       <c r="C127" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11857,7 +11559,6 @@
           <t>王一行</t>
         </is>
       </c>
-      <c r="B128" t="inlineStr"/>
       <c r="C128" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11870,7 +11571,6 @@
           <t>王娇娇</t>
         </is>
       </c>
-      <c r="B129" t="inlineStr"/>
       <c r="C129" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11883,7 +11583,6 @@
           <t>王睿龙</t>
         </is>
       </c>
-      <c r="B130" t="inlineStr"/>
       <c r="C130" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11896,7 +11595,6 @@
           <t>王袆哲</t>
         </is>
       </c>
-      <c r="B131" t="inlineStr"/>
       <c r="C131" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11909,7 +11607,6 @@
           <t>石天奇</t>
         </is>
       </c>
-      <c r="B132" t="inlineStr"/>
       <c r="C132" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11922,7 +11619,6 @@
           <t>石晨露</t>
         </is>
       </c>
-      <c r="B133" t="inlineStr"/>
       <c r="C133" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11935,7 +11631,6 @@
           <t>石英杰</t>
         </is>
       </c>
-      <c r="B134" t="inlineStr"/>
       <c r="C134" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11948,7 +11643,6 @@
           <t>罗帅杰</t>
         </is>
       </c>
-      <c r="B135" t="inlineStr"/>
       <c r="C135" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11961,7 +11655,6 @@
           <t>菜娇阳</t>
         </is>
       </c>
-      <c r="B136" t="inlineStr"/>
       <c r="C136" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11974,7 +11667,6 @@
           <t>蔡晨阳</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr"/>
       <c r="C137" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -11987,7 +11679,6 @@
           <t>蔡芷茵</t>
         </is>
       </c>
-      <c r="B138" t="inlineStr"/>
       <c r="C138" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -12000,7 +11691,6 @@
           <t>裴炬米</t>
         </is>
       </c>
-      <c r="B139" t="inlineStr"/>
       <c r="C139" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -12013,7 +11703,6 @@
           <t>赵佳谊</t>
         </is>
       </c>
-      <c r="B140" t="inlineStr"/>
       <c r="C140" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -12026,7 +11715,6 @@
           <t>赵天皓</t>
         </is>
       </c>
-      <c r="B141" t="inlineStr"/>
       <c r="C141" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -12039,7 +11727,6 @@
           <t>赵晟煜</t>
         </is>
       </c>
-      <c r="B142" t="inlineStr"/>
       <c r="C142" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -12052,7 +11739,6 @@
           <t>赵熙宁</t>
         </is>
       </c>
-      <c r="B143" t="inlineStr"/>
       <c r="C143" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -12065,7 +11751,6 @@
           <t>郭佳怡</t>
         </is>
       </c>
-      <c r="B144" t="inlineStr"/>
       <c r="C144" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -12078,7 +11763,6 @@
           <t>郭佳煜</t>
         </is>
       </c>
-      <c r="B145" t="inlineStr"/>
       <c r="C145" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -12091,7 +11775,6 @@
           <t>郭家硕</t>
         </is>
       </c>
-      <c r="B146" t="inlineStr"/>
       <c r="C146" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -12104,7 +11787,6 @@
           <t>郭文昊</t>
         </is>
       </c>
-      <c r="B147" t="inlineStr"/>
       <c r="C147" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -12117,7 +11799,6 @@
           <t>郭昊航</t>
         </is>
       </c>
-      <c r="B148" t="inlineStr"/>
       <c r="C148" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -12130,7 +11811,6 @@
           <t>郭瑞洁</t>
         </is>
       </c>
-      <c r="B149" t="inlineStr"/>
       <c r="C149" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -12143,7 +11823,6 @@
           <t>靳志科</t>
         </is>
       </c>
-      <c r="B150" t="inlineStr"/>
       <c r="C150" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -12156,7 +11835,6 @@
           <t>马祥瑞</t>
         </is>
       </c>
-      <c r="B151" t="inlineStr"/>
       <c r="C151" t="inlineStr">
         <is>
           <t>高中同学</t>
@@ -12271,7 +11949,6 @@
           <t>何思嘉</t>
         </is>
       </c>
-      <c r="B158" t="inlineStr"/>
       <c r="C158" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -12284,7 +11961,6 @@
           <t>何淑贤</t>
         </is>
       </c>
-      <c r="B159" t="inlineStr"/>
       <c r="C159" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -12314,7 +11990,6 @@
           <t>冯政锡</t>
         </is>
       </c>
-      <c r="B161" t="inlineStr"/>
       <c r="C161" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -12565,7 +12240,6 @@
           <t>宋晓格</t>
         </is>
       </c>
-      <c r="B176" t="inlineStr"/>
       <c r="C176" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -12714,7 +12388,6 @@
           <t>张紫轩</t>
         </is>
       </c>
-      <c r="B185" t="inlineStr"/>
       <c r="C185" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -12761,7 +12434,6 @@
           <t>徐畅</t>
         </is>
       </c>
-      <c r="B188" t="inlineStr"/>
       <c r="C188" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -12808,7 +12480,6 @@
           <t>曹鹏威</t>
         </is>
       </c>
-      <c r="B191" t="inlineStr"/>
       <c r="C191" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -12821,7 +12492,6 @@
           <t>李俊谣</t>
         </is>
       </c>
-      <c r="B192" t="inlineStr"/>
       <c r="C192" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -12834,7 +12504,6 @@
           <t>李华婷</t>
         </is>
       </c>
-      <c r="B193" t="inlineStr"/>
       <c r="C193" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -12847,7 +12516,6 @@
           <t>李小芝</t>
         </is>
       </c>
-      <c r="B194" t="inlineStr"/>
       <c r="C194" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -12877,7 +12545,6 @@
           <t>李文浩</t>
         </is>
       </c>
-      <c r="B196" t="inlineStr"/>
       <c r="C196" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -12924,7 +12591,6 @@
           <t>李瑞豪</t>
         </is>
       </c>
-      <c r="B199" t="inlineStr"/>
       <c r="C199" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -12954,7 +12620,6 @@
           <t>李鑫茹</t>
         </is>
       </c>
-      <c r="B201" t="inlineStr"/>
       <c r="C201" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -13052,7 +12717,6 @@
           <t>梁其燕</t>
         </is>
       </c>
-      <c r="B207" t="inlineStr"/>
       <c r="C207" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -13116,7 +12780,6 @@
           <t>王宗彭</t>
         </is>
       </c>
-      <c r="B211" t="inlineStr"/>
       <c r="C211" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -13248,7 +12911,6 @@
           <t>田梦瑶</t>
         </is>
       </c>
-      <c r="B219" t="inlineStr"/>
       <c r="C219" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -13363,7 +13025,6 @@
           <t>肖梦凯</t>
         </is>
       </c>
-      <c r="B226" t="inlineStr"/>
       <c r="C226" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -13376,7 +13037,6 @@
           <t>胡巧熠</t>
         </is>
       </c>
-      <c r="B227" t="inlineStr"/>
       <c r="C227" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -13508,7 +13168,6 @@
           <t>袁烁</t>
         </is>
       </c>
-      <c r="B235" t="inlineStr"/>
       <c r="C235" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -13521,7 +13180,6 @@
           <t>谢圣教</t>
         </is>
       </c>
-      <c r="B236" t="inlineStr"/>
       <c r="C236" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -13551,7 +13209,6 @@
           <t>赵毅</t>
         </is>
       </c>
-      <c r="B238" t="inlineStr"/>
       <c r="C238" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -13734,7 +13391,6 @@
           <t>郭琳</t>
         </is>
       </c>
-      <c r="B249" t="inlineStr"/>
       <c r="C249" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -13747,7 +13403,6 @@
           <t>闫泽宇</t>
         </is>
       </c>
-      <c r="B250" t="inlineStr"/>
       <c r="C250" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -13760,7 +13415,6 @@
           <t>陈卓</t>
         </is>
       </c>
-      <c r="B251" t="inlineStr"/>
       <c r="C251" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -13790,7 +13444,6 @@
           <t>陈广凤</t>
         </is>
       </c>
-      <c r="B253" t="inlineStr"/>
       <c r="C253" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -13973,7 +13626,6 @@
           <t>高彤</t>
         </is>
       </c>
-      <c r="B264" t="inlineStr"/>
       <c r="C264" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -14020,7 +13672,6 @@
           <t>鲁静</t>
         </is>
       </c>
-      <c r="B267" t="inlineStr"/>
       <c r="C267" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -14033,7 +13684,6 @@
           <t>黄泽豪</t>
         </is>
       </c>
-      <c r="B268" t="inlineStr"/>
       <c r="C268" t="inlineStr">
         <is>
           <t>大学同学</t>
@@ -14097,7 +13747,6 @@
           <t>侯胜利</t>
         </is>
       </c>
-      <c r="B272" t="inlineStr"/>
       <c r="C272" t="inlineStr">
         <is>
           <t>大学老师</t>
@@ -14110,7 +13759,6 @@
           <t>刘莹莹</t>
         </is>
       </c>
-      <c r="B273" t="inlineStr"/>
       <c r="C273" t="inlineStr">
         <is>
           <t>高中老师</t>
@@ -14123,7 +13771,6 @@
           <t>卫莉莉</t>
         </is>
       </c>
-      <c r="B274" t="inlineStr"/>
       <c r="C274" t="inlineStr">
         <is>
           <t>大学老师</t>
@@ -14136,7 +13783,6 @@
           <t>吴程浩</t>
         </is>
       </c>
-      <c r="B275" t="inlineStr"/>
       <c r="C275" t="inlineStr">
         <is>
           <t>大学老师</t>
@@ -14149,7 +13795,6 @@
           <t>吴艳娜</t>
         </is>
       </c>
-      <c r="B276" t="inlineStr"/>
       <c r="C276" t="inlineStr">
         <is>
           <t>初中老师</t>
@@ -14162,7 +13807,6 @@
           <t>周家全</t>
         </is>
       </c>
-      <c r="B277" t="inlineStr"/>
       <c r="C277" t="inlineStr">
         <is>
           <t>大学老师</t>
@@ -14175,7 +13819,6 @@
           <t>姚华平</t>
         </is>
       </c>
-      <c r="B278" t="inlineStr"/>
       <c r="C278" t="inlineStr">
         <is>
           <t>大学老师</t>
@@ -14188,7 +13831,6 @@
           <t>张文娟</t>
         </is>
       </c>
-      <c r="B279" t="inlineStr"/>
       <c r="C279" t="inlineStr">
         <is>
           <t>初中老师</t>
@@ -14201,7 +13843,6 @@
           <t>张景燕</t>
         </is>
       </c>
-      <c r="B280" t="inlineStr"/>
       <c r="C280" t="inlineStr">
         <is>
           <t>初中老师</t>
@@ -14214,7 +13855,6 @@
           <t>张荣</t>
         </is>
       </c>
-      <c r="B281" t="inlineStr"/>
       <c r="C281" t="inlineStr">
         <is>
           <t>大学老师</t>
@@ -14227,7 +13867,6 @@
           <t>张豪</t>
         </is>
       </c>
-      <c r="B282" t="inlineStr"/>
       <c r="C282" t="inlineStr">
         <is>
           <t>大学老师</t>
@@ -14240,7 +13879,6 @@
           <t>张靖波</t>
         </is>
       </c>
-      <c r="B283" t="inlineStr"/>
       <c r="C283" t="inlineStr">
         <is>
           <t>初中老师</t>
@@ -14253,7 +13891,6 @@
           <t>徐键</t>
         </is>
       </c>
-      <c r="B284" t="inlineStr"/>
       <c r="C284" t="inlineStr">
         <is>
           <t>高中老师</t>
@@ -14266,7 +13903,6 @@
           <t>李志先</t>
         </is>
       </c>
-      <c r="B285" t="inlineStr"/>
       <c r="C285" t="inlineStr">
         <is>
           <t>大学老师</t>
@@ -14279,7 +13915,6 @@
           <t>李明照</t>
         </is>
       </c>
-      <c r="B286" t="inlineStr"/>
       <c r="C286" t="inlineStr">
         <is>
           <t>大学老师</t>
@@ -14292,7 +13927,6 @@
           <t>李晓光</t>
         </is>
       </c>
-      <c r="B287" t="inlineStr"/>
       <c r="C287" t="inlineStr">
         <is>
           <t>大学老师</t>
@@ -14305,7 +13939,6 @@
           <t>李晨</t>
         </is>
       </c>
-      <c r="B288" t="inlineStr"/>
       <c r="C288" t="inlineStr">
         <is>
           <t>大学老师</t>
@@ -14318,7 +13951,6 @@
           <t>杨向兰</t>
         </is>
       </c>
-      <c r="B289" t="inlineStr"/>
       <c r="C289" t="inlineStr">
         <is>
           <t>大学老师</t>
@@ -14331,7 +13963,6 @@
           <t>梁培霞</t>
         </is>
       </c>
-      <c r="B290" t="inlineStr"/>
       <c r="C290" t="inlineStr">
         <is>
           <t>初中老师</t>
@@ -14344,7 +13975,6 @@
           <t>梁雪华</t>
         </is>
       </c>
-      <c r="B291" t="inlineStr"/>
       <c r="C291" t="inlineStr">
         <is>
           <t>大学老师</t>
@@ -14357,7 +13987,6 @@
           <t>樊玉荣</t>
         </is>
       </c>
-      <c r="B292" t="inlineStr"/>
       <c r="C292" t="inlineStr">
         <is>
           <t>初中老师</t>
@@ -14370,7 +13999,6 @@
           <t>王亚钰</t>
         </is>
       </c>
-      <c r="B293" t="inlineStr"/>
       <c r="C293" t="inlineStr">
         <is>
           <t>大学老师</t>
@@ -14383,7 +14011,6 @@
           <t>王志强</t>
         </is>
       </c>
-      <c r="B294" t="inlineStr"/>
       <c r="C294" t="inlineStr">
         <is>
           <t>高中老师</t>
@@ -14396,7 +14023,6 @@
           <t>王海滨</t>
         </is>
       </c>
-      <c r="B295" t="inlineStr"/>
       <c r="C295" t="inlineStr">
         <is>
           <t>高中老师</t>
@@ -14409,7 +14035,6 @@
           <t>王淑萍</t>
         </is>
       </c>
-      <c r="B296" t="inlineStr"/>
       <c r="C296" t="inlineStr">
         <is>
           <t>初中老师</t>
@@ -14422,7 +14047,6 @@
           <t>石青岩</t>
         </is>
       </c>
-      <c r="B297" t="inlineStr"/>
       <c r="C297" t="inlineStr">
         <is>
           <t>高中老师</t>
@@ -14435,7 +14059,6 @@
           <t>童新安</t>
         </is>
       </c>
-      <c r="B298" t="inlineStr"/>
       <c r="C298" t="inlineStr">
         <is>
           <t>大学老师</t>
@@ -14448,7 +14071,6 @@
           <t>肖惠朝</t>
         </is>
       </c>
-      <c r="B299" t="inlineStr"/>
       <c r="C299" t="inlineStr">
         <is>
           <t>大学老师</t>
@@ -14461,7 +14083,6 @@
           <t>苏秀燕</t>
         </is>
       </c>
-      <c r="B300" t="inlineStr"/>
       <c r="C300" t="inlineStr">
         <is>
           <t>高中老师</t>
@@ -14474,7 +14095,6 @@
           <t>蒋芳</t>
         </is>
       </c>
-      <c r="B301" t="inlineStr"/>
       <c r="C301" t="inlineStr">
         <is>
           <t>初中老师</t>
@@ -14487,7 +14107,6 @@
           <t>许超</t>
         </is>
       </c>
-      <c r="B302" t="inlineStr"/>
       <c r="C302" t="inlineStr">
         <is>
           <t>大学老师</t>
@@ -14500,7 +14119,6 @@
           <t>赵春山</t>
         </is>
       </c>
-      <c r="B303" t="inlineStr"/>
       <c r="C303" t="inlineStr">
         <is>
           <t>高中老师</t>
@@ -14513,7 +14131,6 @@
           <t>郑卫东</t>
         </is>
       </c>
-      <c r="B304" t="inlineStr"/>
       <c r="C304" t="inlineStr">
         <is>
           <t>大学老师</t>
@@ -14526,7 +14143,6 @@
           <t>郑志伟</t>
         </is>
       </c>
-      <c r="B305" t="inlineStr"/>
       <c r="C305" t="inlineStr">
         <is>
           <t>高中老师</t>
@@ -14539,7 +14155,6 @@
           <t>郭玉珂</t>
         </is>
       </c>
-      <c r="B306" t="inlineStr"/>
       <c r="C306" t="inlineStr">
         <is>
           <t>大学老师</t>
@@ -14552,7 +14167,6 @@
           <t>郭素霞</t>
         </is>
       </c>
-      <c r="B307" t="inlineStr"/>
       <c r="C307" t="inlineStr">
         <is>
           <t>初中老师</t>
@@ -14565,7 +14179,6 @@
           <t>郭红宇</t>
         </is>
       </c>
-      <c r="B308" t="inlineStr"/>
       <c r="C308" t="inlineStr">
         <is>
           <t>初中老师</t>
@@ -14578,7 +14191,6 @@
           <t>钱素娥</t>
         </is>
       </c>
-      <c r="B309" t="inlineStr"/>
       <c r="C309" t="inlineStr">
         <is>
           <t>初中老师</t>
@@ -14591,7 +14203,6 @@
           <t>陈向瑞</t>
         </is>
       </c>
-      <c r="B310" t="inlineStr"/>
       <c r="C310" t="inlineStr">
         <is>
           <t>高中老师</t>
@@ -14604,7 +14215,6 @@
           <t>陶荣</t>
         </is>
       </c>
-      <c r="B311" t="inlineStr"/>
       <c r="C311" t="inlineStr">
         <is>
           <t>大学老师</t>
@@ -14617,7 +14227,6 @@
           <t>韩婧斐</t>
         </is>
       </c>
-      <c r="B312" t="inlineStr"/>
       <c r="C312" t="inlineStr">
         <is>
           <t>高中老师</t>
@@ -14630,7 +14239,6 @@
           <t>韩斌</t>
         </is>
       </c>
-      <c r="B313" t="inlineStr"/>
       <c r="C313" t="inlineStr">
         <is>
           <t>高中老师</t>
@@ -14643,7 +14251,6 @@
           <t>骆正玉</t>
         </is>
       </c>
-      <c r="B314" t="inlineStr"/>
       <c r="C314" t="inlineStr">
         <is>
           <t>初中老师</t>
@@ -14656,7 +14263,6 @@
           <t>高春玲</t>
         </is>
       </c>
-      <c r="B315" t="inlineStr"/>
       <c r="C315" t="inlineStr">
         <is>
           <t>大学老师</t>
@@ -14669,7 +14275,6 @@
           <t>魏玉堂</t>
         </is>
       </c>
-      <c r="B316" t="inlineStr"/>
       <c r="C316" t="inlineStr">
         <is>
           <t>高中老师</t>
@@ -14682,7 +14287,6 @@
           <t>龚蕾</t>
         </is>
       </c>
-      <c r="B317" t="inlineStr"/>
       <c r="C317" t="inlineStr">
         <is>
           <t>大学老师</t>
@@ -14700,7 +14304,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -14794,50 +14398,34 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>大学生暑期"三下乡"支教活动</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr"/>
+          <t>摇滚马拉松志愿者证书</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>/static/uploads/events/1faee366999443f79f0c939d6128bf6d.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>摇滚马拉松志愿者证书</t>
+          <t>校园马拉松 一等奖</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>/static/uploads/events/1faee366999443f79f0c939d6128bf6d.jpg</t>
+          <t>/static/uploads/events/75c0d946fe2546f88768516e33044828.jpg</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>校园马拉松 一等奖</t>
+          <t>美国大学生数学建模竞赛H奖</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
-        <is>
-          <t>/static/uploads/events/75c0d946fe2546f88768516e33044828.jpg</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>洛阳2024摇滚马拉松</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr"/>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>美国大学生数学建模竞赛H奖</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
         <is>
           <t>/static/uploads/events/d1129f3176674b7b89d60bcaf0fc2ed5.png</t>
         </is>
@@ -14949,7 +14537,6 @@
 训练与导出：PyTorch 训练（断点续训、Early Stopping）→ ONNX 导出并部署到 Android</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -14991,7 +14578,6 @@
 设置：深色/浅色主题、中英文界面、设置持久化</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -15034,7 +14620,6 @@
 后端：模块化 Flask、健康检查、错误收集、服务监控</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15078,7 +14663,6 @@
           <t>100%鲜橙汁</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
       <c r="C2" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15108,7 +14692,6 @@
           <t>FLORENCE</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
       <c r="C4" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15121,7 +14704,6 @@
           <t>JADED</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
       <c r="C5" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15134,7 +14716,6 @@
           <t>LoveChoice 捡爱</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
       <c r="C6" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15147,7 +14728,6 @@
           <t>PEAK</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
       <c r="C7" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15177,7 +14757,6 @@
           <t>Sizeable</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15190,7 +14769,6 @@
           <t>The Wanderer: Frankenstein's Creature</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
       <c r="C10" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15203,7 +14781,6 @@
           <t>不巷歌</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
       <c r="C11" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15216,7 +14793,6 @@
           <t>人类一败涂地</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
       <c r="C12" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15229,7 +14805,6 @@
           <t>传说之下</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr"/>
       <c r="C13" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15327,7 +14902,6 @@
           <t>冰与火之舞</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr"/>
       <c r="C19" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15391,7 +14965,6 @@
           <t>前方高能</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr"/>
       <c r="C23" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15404,7 +14977,6 @@
           <t>历历在目</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr"/>
       <c r="C24" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15417,7 +14989,6 @@
           <t>原子之心</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
       <c r="C25" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15430,7 +15001,6 @@
           <t>去月球</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15443,7 +15013,6 @@
           <t>双人成行</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
       <c r="C27" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15456,7 +15025,6 @@
           <t>地狱边境</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr"/>
       <c r="C28" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15486,7 +15054,6 @@
           <t>塔罗斯的法则</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr"/>
       <c r="C30" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15499,7 +15066,6 @@
           <t>墨池镇</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr"/>
       <c r="C31" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15512,7 +15078,6 @@
           <t>多重花园</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr"/>
       <c r="C32" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15525,7 +15090,6 @@
           <t>夺蛋骑兵</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr"/>
       <c r="C33" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15538,7 +15102,6 @@
           <t>孤山独影</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr"/>
       <c r="C34" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15551,7 +15114,6 @@
           <t>孤帆远航</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr"/>
       <c r="C35" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15564,7 +15126,6 @@
           <t>密码</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr"/>
       <c r="C36" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15577,7 +15138,6 @@
           <t>寻找天堂</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr"/>
       <c r="C37" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15590,7 +15150,6 @@
           <t>山谷</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15603,7 +15162,6 @@
           <t>崩溃大陆</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr"/>
       <c r="C39" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15616,7 +15174,6 @@
           <t>巫师3：狂猎</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15629,7 +15186,6 @@
           <t>巴别塔圣歌</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr"/>
       <c r="C41" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15642,7 +15198,6 @@
           <t>师父</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr"/>
       <c r="C42" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15655,7 +15210,6 @@
           <t>幽灵行者</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15668,7 +15222,6 @@
           <t>异星装置博物馆</t>
         </is>
       </c>
-      <c r="B44" t="inlineStr"/>
       <c r="C44" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15681,7 +15234,6 @@
           <t>影子工厂</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15694,7 +15246,6 @@
           <t>德州电锯杀人狂</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15707,7 +15258,6 @@
           <t>我们也在这里</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15720,7 +15270,6 @@
           <t>我是僵尸</t>
         </is>
       </c>
-      <c r="B48" t="inlineStr"/>
       <c r="C48" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15733,7 +15282,6 @@
           <t>我的世界：传奇</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr"/>
       <c r="C49" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15780,7 +15328,6 @@
           <t>战锤40K：格雷迪厄斯-遗迹之战</t>
         </is>
       </c>
-      <c r="B52" t="inlineStr"/>
       <c r="C52" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15827,7 +15374,6 @@
           <t>拉娜的星球</t>
         </is>
       </c>
-      <c r="B55" t="inlineStr"/>
       <c r="C55" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15908,7 +15454,6 @@
           <t>无尽传奇</t>
         </is>
       </c>
-      <c r="B60" t="inlineStr"/>
       <c r="C60" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15921,7 +15466,6 @@
           <t>星际小队</t>
         </is>
       </c>
-      <c r="B61" t="inlineStr"/>
       <c r="C61" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15934,7 +15478,6 @@
           <t>星露谷物语</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15947,7 +15490,6 @@
           <t>暴雨</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr"/>
       <c r="C63" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -15960,7 +15502,6 @@
           <t>最后的篝火</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr"/>
       <c r="C64" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16007,7 +15548,6 @@
           <t>极限国度</t>
         </is>
       </c>
-      <c r="B67" t="inlineStr"/>
       <c r="C67" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16020,7 +15560,6 @@
           <t>森林</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16067,7 +15606,6 @@
           <t>死亡细胞</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16080,7 +15618,6 @@
           <t>求生之路2</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr"/>
       <c r="C72" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16093,7 +15630,6 @@
           <t>泰坦陨落2</t>
         </is>
       </c>
-      <c r="B73" t="inlineStr"/>
       <c r="C73" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16106,7 +15642,6 @@
           <t>泰拉瑞亚</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16119,7 +15654,6 @@
           <t>海浪物语</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr"/>
       <c r="C75" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16132,7 +15666,6 @@
           <t>消逝的光芒</t>
         </is>
       </c>
-      <c r="B76" t="inlineStr"/>
       <c r="C76" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16145,7 +15678,6 @@
           <t>深入</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16158,7 +15690,6 @@
           <t>火山的女儿</t>
         </is>
       </c>
-      <c r="B78" t="inlineStr"/>
       <c r="C78" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16171,7 +15702,6 @@
           <t>灰色</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr"/>
       <c r="C79" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16184,7 +15714,6 @@
           <t>灵异校园</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr"/>
       <c r="C80" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16197,7 +15726,6 @@
           <t>灵魂摆渡人</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr"/>
       <c r="C81" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16244,7 +15772,6 @@
           <t>王国：两位君主</t>
         </is>
       </c>
-      <c r="B84" t="inlineStr"/>
       <c r="C84" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16257,7 +15784,6 @@
           <t>甜甜圈都市</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr"/>
       <c r="C85" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16270,7 +15796,6 @@
           <t>画中世界</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr"/>
       <c r="C86" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16283,7 +15808,6 @@
           <t>白色阴影</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr"/>
       <c r="C87" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16313,7 +15837,6 @@
           <t>盛夏盛开的花</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr"/>
       <c r="C89" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16394,7 +15917,6 @@
           <t>精灵与萤火意志</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr"/>
       <c r="C94" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16526,7 +16048,6 @@
           <t>脑叶公司 | 模拟怪物管理</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr"/>
       <c r="C102" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16539,7 +16060,6 @@
           <t>至暗时刻</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr"/>
       <c r="C103" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16552,7 +16072,6 @@
           <t>艾迪芬奇的记忆</t>
         </is>
       </c>
-      <c r="B104" t="inlineStr"/>
       <c r="C104" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16565,7 +16084,6 @@
           <t>荒野大镖客：救赎2</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr"/>
       <c r="C105" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16578,7 +16096,6 @@
           <t>蔚蓝</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr"/>
       <c r="C106" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16642,7 +16159,6 @@
           <t>行尸走肉：终极系列合集</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr"/>
       <c r="C110" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16655,7 +16171,6 @@
           <t>见证者</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr"/>
       <c r="C111" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16668,7 +16183,6 @@
           <t>诡计穿越僵尸末日</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr"/>
       <c r="C112" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16681,7 +16195,6 @@
           <t>逃生：试炼</t>
         </is>
       </c>
-      <c r="B113" t="inlineStr"/>
       <c r="C113" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16694,7 +16207,6 @@
           <t>逃离后室</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr"/>
       <c r="C114" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16741,7 +16253,6 @@
           <t>链在一起</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr"/>
       <c r="C117" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16754,7 +16265,6 @@
           <t>随从大师</t>
         </is>
       </c>
-      <c r="B118" t="inlineStr"/>
       <c r="C118" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16767,7 +16277,6 @@
           <t>雨中冒险2</t>
         </is>
       </c>
-      <c r="B119" t="inlineStr"/>
       <c r="C119" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16780,7 +16289,6 @@
           <t>霍格沃兹之遗</t>
         </is>
       </c>
-      <c r="B120" t="inlineStr"/>
       <c r="C120" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16793,7 +16301,6 @@
           <t>风之旅人</t>
         </is>
       </c>
-      <c r="B121" t="inlineStr"/>
       <c r="C121" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16806,7 +16313,6 @@
           <t>饥荒</t>
         </is>
       </c>
-      <c r="B122" t="inlineStr"/>
       <c r="C122" t="inlineStr">
         <is>
           <t>Steam</t>
@@ -16819,7 +16325,6 @@
           <t>Garden Story</t>
         </is>
       </c>
-      <c r="B123" t="inlineStr"/>
       <c r="C123" t="inlineStr">
         <is>
           <t>Epic</t>
@@ -16832,7 +16337,6 @@
           <t>僵尸世界大战：劫后余生</t>
         </is>
       </c>
-      <c r="B124" t="inlineStr"/>
       <c r="C124" t="inlineStr">
         <is>
           <t>Epic</t>
@@ -16845,7 +16349,6 @@
           <t>取景器</t>
         </is>
       </c>
-      <c r="B125" t="inlineStr"/>
       <c r="C125" t="inlineStr">
         <is>
           <t>Epic</t>
@@ -16858,7 +16361,6 @@
           <t>彩虹小马格斗</t>
         </is>
       </c>
-      <c r="B126" t="inlineStr"/>
       <c r="C126" t="inlineStr">
         <is>
           <t>Epic</t>
@@ -16871,7 +16373,6 @@
           <t>我们一起在这里</t>
         </is>
       </c>
-      <c r="B127" t="inlineStr"/>
       <c r="C127" t="inlineStr">
         <is>
           <t>Epic</t>
@@ -16884,7 +16385,6 @@
           <t>无人愿死</t>
         </is>
       </c>
-      <c r="B128" t="inlineStr"/>
       <c r="C128" t="inlineStr">
         <is>
           <t>Epic</t>
@@ -16897,7 +16397,6 @@
           <t>黑暗侦探：黑暗中的摸索</t>
         </is>
       </c>
-      <c r="B129" t="inlineStr"/>
       <c r="C129" t="inlineStr">
         <is>
           <t>Epic</t>

</xml_diff>

<commit_message>
Update books spreadsheet and regenerate export list
Remove web-novel-only entries from zhita_settings and sync 书籍.txt export.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/zhita_settings.xlsx
+++ b/zhita_settings.xlsx
@@ -8223,7 +8223,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C94"/>
+  <dimension ref="A1:C67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -8251,29 +8251,29 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>HMI专业催眠师教程</t>
+          <t>书名</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>专业教材</t>
+          <t>作者</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>实体书</t>
+          <t>分类</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>一个陌生女人的来信</t>
+          <t>HMI专业催眠师教程</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>斯蒂芬·茨威格</t>
+          <t>专业教材</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8285,12 +8285,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>三体</t>
+          <t>一个陌生女人的来信</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>刘慈欣</t>
+          <t>斯蒂芬·茨威格</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -8302,12 +8302,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>三重门</t>
+          <t>三体</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>韩寒</t>
+          <t>刘慈欣</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -8319,12 +8319,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>下一站,天国</t>
+          <t>三重门</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>是枝裕和</t>
+          <t>韩寒</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -8336,12 +8336,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>不正常人类症候群</t>
+          <t>下一站,天国</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>张寒寺</t>
+          <t>是枝裕和</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -8353,12 +8353,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>不要挑战人性</t>
+          <t>不正常人类症候群</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>邓娟</t>
+          <t>张寒寺</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -8370,46 +8370,46 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>世界上最神奇的60个经典定律</t>
+          <t>不要挑战人性</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>张新国</t>
+          <t>邓娟</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>网文</t>
+          <t>实体书</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>云边有个小卖部</t>
+          <t>世界上最神奇的60个经典定律</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>张嘉佳</t>
+          <t>张新国</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>实体书</t>
+          <t>网文</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>人间失格</t>
+          <t>云边有个小卖部</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>太宰治</t>
+          <t>张嘉佳</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -8421,17 +8421,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>他悄悄地亲吻过</t>
+          <t>人间失格</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>网文作者</t>
+          <t>太宰治</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>网文</t>
+          <t>实体书</t>
         </is>
       </c>
     </row>
@@ -8506,46 +8506,46 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>全球通缉：疯了！你管这个叫逃亡</t>
+          <t>全球高考</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>网文作者</t>
+          <t>木苏里</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>网文</t>
+          <t>实体书与网文</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>全球高考</t>
+          <t>区块链</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>木苏里</t>
+          <t>专业书籍</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>实体书与网文</t>
+          <t>实体书</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>区块链</t>
+          <t>古都</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>专业书籍</t>
+          <t>川端康成</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -8557,12 +8557,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>古都</t>
+          <t>呼啸山庄</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>川端康成</t>
+          <t>艾米莉·勃朗特</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -8574,29 +8574,29 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>向来凉薄，何言情深</t>
+          <t>哈佛家训</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>网文作者</t>
+          <t>威廉·贝纳德</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>网文</t>
+          <t>实体书</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>呼啸山庄</t>
+          <t>地下室手记</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>艾米莉·勃朗特</t>
+          <t>陀思妥耶夫斯基</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -8608,29 +8608,29 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>哈佛家训</t>
+          <t>地球无应答</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>威廉·贝纳德</t>
+          <t>王诺诺</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>实体书</t>
+          <t>网文</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>地下室手记</t>
+          <t>坍缩</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>陀思妥耶夫斯基</t>
+          <t>刘慈欣</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -8642,46 +8642,46 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>地球无应答</t>
+          <t>夏天、烟火和我的尸体</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>王诺诺</t>
+          <t>乙一</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>网文</t>
+          <t>实体书</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>坍缩</t>
+          <t>天官赐福</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>刘慈欣</t>
+          <t>墨香铜臭</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>实体书</t>
+          <t>实体书与网文</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>夏天、烟火和我的尸体</t>
+          <t>天才在左疯子在右：心理疾病漫谈</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>乙一</t>
+          <t>高铭</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -8693,29 +8693,29 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>天官赐福</t>
+          <t>天气之子</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>墨香铜臭</t>
+          <t>新海诚</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>实体书与网文</t>
+          <t>实体书</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>天才在左疯子在右：心理疾病漫谈</t>
+          <t>女儿红</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>高铭</t>
+          <t>简媜</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -8727,12 +8727,12 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>天气之子</t>
+          <t>嫌疑人X的献身</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>新海诚</t>
+          <t>东野圭吾</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -8744,29 +8744,29 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>天降系女友是可爱富婆</t>
+          <t>完美人设</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>网文作者</t>
+          <t>和田秀树</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>网文</t>
+          <t>实体书</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>女儿红</t>
+          <t>小王子</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>简媜</t>
+          <t>安托万·德·圣-埃克苏佩里</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -8778,24 +8778,24 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>女朋友患有渴肤症是种什么体验</t>
+          <t>局外人</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>网文作者</t>
+          <t>阿尔贝·加缪</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>网文</t>
+          <t>实体书</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>好烦啊，高冷校花天天倒追我</t>
+          <t>异草奇花</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -8812,12 +8812,12 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>嫌疑人X的献身</t>
+          <t>很杂很杂的杂学知识</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>东野圭吾</t>
+          <t>张朝元</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -8829,12 +8829,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>完美人设</t>
+          <t>悟空传</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>和田秀树</t>
+          <t>今何在</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -8846,12 +8846,12 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>小王子</t>
+          <t>我是猫</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>安托万·德·圣-埃克苏佩里</t>
+          <t>夏目漱石</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -8863,12 +8863,12 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>局外人</t>
+          <t>挪威的森林</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>阿尔贝·加缪</t>
+          <t>村上春树</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -8880,46 +8880,46 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>开局被校花表白？</t>
+          <t>文城</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>网文作者</t>
+          <t>余华</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>网文</t>
+          <t>实体书</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>异草奇花</t>
+          <t>斯坦福高效睡眠法</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>网文作者</t>
+          <t>西野精治</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>网文</t>
+          <t>实体书</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>很杂很杂的杂学知识</t>
+          <t>月亮与六便士</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>张朝元</t>
+          <t>毛姆</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -8931,46 +8931,46 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>急！合租女友太可爱了怎么办？！</t>
+          <t>某某</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>网文作者</t>
+          <t>木苏里</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>网文</t>
+          <t>实体书与网文</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>恋爱养成：我家老婆太可爱了！</t>
+          <t>水问</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>网文作者</t>
+          <t>简媜</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>网文</t>
+          <t>实体书</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>悟空传</t>
+          <t>海底两万里</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>今何在</t>
+          <t>儒勒·凡尔纳</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -8982,29 +8982,29 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>憨憨同桌傻白甜，把她聊成小女友</t>
+          <t>海边的卡夫卡</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>网文作者</t>
+          <t>村上春树</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>网文</t>
+          <t>实体书</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>我是猫</t>
+          <t>痴人之爱</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>夏目漱石</t>
+          <t>谷崎润一郎</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -9016,29 +9016,29 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>我的老婆怎么能这么可爱？</t>
+          <t>白夜</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>网文作者</t>
+          <t>陀思妥耶夫斯基</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>网文</t>
+          <t>实体书</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>挪威的森林</t>
+          <t>白夜行</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>村上春树</t>
+          <t>东野圭吾</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -9050,29 +9050,29 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>摔了一跤后，我决定不矜持了</t>
+          <t>白金数据</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>网文作者</t>
+          <t>东野圭吾</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>网文</t>
+          <t>实体书</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>文城</t>
+          <t>百年孤独</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>余华</t>
+          <t>加西亚·马尔克斯</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -9084,12 +9084,12 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>斯坦福高效睡眠法</t>
+          <t>睡美人</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>西野精治</t>
+          <t>川端康成</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -9101,12 +9101,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>月亮与六便士</t>
+          <t>窄门</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>毛姆</t>
+          <t>安德烈·纪德</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -9118,29 +9118,29 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>某某</t>
+          <t>简爱</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>木苏里</t>
+          <t>夏洛蒂·勃朗特</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>实体书与网文</t>
+          <t>实体书</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>水问</t>
+          <t>红与黑</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>简媜</t>
+          <t>司汤达</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -9152,29 +9152,29 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>沈少，夫人重生后哭着要以身相许</t>
+          <t>罗生门</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>网文作者</t>
+          <t>芥川龙之介</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>网文</t>
+          <t>实体书</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>海底两万里</t>
+          <t>罪与罚</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>儒勒·凡尔纳</t>
+          <t>陀思妥耶夫斯基</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -9186,12 +9186,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>海边的卡夫卡</t>
+          <t>老人与海</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>村上春树</t>
+          <t>欧内斯特·海明威</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -9203,29 +9203,29 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>玫瑰冠冕</t>
+          <t>胭脂盆地</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>网文作者</t>
+          <t>简媜</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>网文</t>
+          <t>实体书</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>痴人之爱</t>
+          <t>自学大全</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>谷崎润一郎</t>
+          <t>读书猴</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -9237,12 +9237,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>白夜</t>
+          <t>解忧杂货店</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>陀思妥耶夫斯基</t>
+          <t>东野圭吾</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -9254,29 +9254,29 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>白夜行</t>
+          <t>诡秘之主</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>东野圭吾</t>
+          <t>爱潜水的乌贼</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>实体书</t>
+          <t>实体书与网文</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>白金数据</t>
+          <t>边城</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>东野圭吾</t>
+          <t>沈从文</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -9288,24 +9288,24 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>百年孤独</t>
+          <t>道诡异仙</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>加西亚·马尔克斯</t>
+          <t>狐尾的笔</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>实体书</t>
+          <t>网文</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>睡美人</t>
+          <t>雪国</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -9322,12 +9322,12 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>窄门</t>
+          <t>霍乱时期的爱情</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>安德烈·纪德</t>
+          <t>加西亚·马尔克斯</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -9339,493 +9339,34 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>等你抬起头时</t>
+          <t>飘</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>网文作者</t>
+          <t>玛格丽特·米切尔</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>网文</t>
+          <t>实体书</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>简爱</t>
+          <t>骆驼祥子</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>夏洛蒂·勃朗特</t>
+          <t>老舍</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
           <t>实体书</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>红与黑</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>司汤达</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>实体书</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>纯欲青梅花式白给后，我们恋爱了</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>网文作者</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>网文</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" t="inlineStr">
-        <is>
-          <t>罗生门</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>芥川龙之介</t>
-        </is>
-      </c>
-      <c r="C70" t="inlineStr">
-        <is>
-          <t>实体书</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>罪与罚</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>陀思妥耶夫斯基</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>实体书</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" t="inlineStr">
-        <is>
-          <t>老人与海</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>欧内斯特·海明威</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>实体书</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" t="inlineStr">
-        <is>
-          <t>考恋爱不如考第一</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>网文作者</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>网文</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" t="inlineStr">
-        <is>
-          <t>胭脂盆地</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
-        <is>
-          <t>简媜</t>
-        </is>
-      </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>实体书</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
-        <is>
-          <t>自学大全</t>
-        </is>
-      </c>
-      <c r="B75" t="inlineStr">
-        <is>
-          <t>读书猴</t>
-        </is>
-      </c>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>实体书</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" t="inlineStr">
-        <is>
-          <t>裴教授上网课，娇妻意外出镜</t>
-        </is>
-      </c>
-      <c r="B76" t="inlineStr">
-        <is>
-          <t>网文作者</t>
-        </is>
-      </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>网文</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>规则怪谈：我能完美利用规则</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>网文作者</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>网文</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" t="inlineStr">
-        <is>
-          <t>解忧杂货店</t>
-        </is>
-      </c>
-      <c r="B78" t="inlineStr">
-        <is>
-          <t>东野圭吾</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>实体书</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
-        <is>
-          <t>诡秘之主</t>
-        </is>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>爱潜水的乌贼</t>
-        </is>
-      </c>
-      <c r="C79" t="inlineStr">
-        <is>
-          <t>实体书与网文</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" t="inlineStr">
-        <is>
-          <t>趁同桌好乖，赶紧忽悠做老婆</t>
-        </is>
-      </c>
-      <c r="B80" t="inlineStr">
-        <is>
-          <t>网文作者</t>
-        </is>
-      </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>网文</t>
-        </is>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>超甜：甜美总裁姐姐对我图谋不轨</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>网文作者</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>网文</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" t="inlineStr">
-        <is>
-          <t>超级学霸：从低调控分开始！</t>
-        </is>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>网文作者</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>网文</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
-        <is>
-          <t>边城</t>
-        </is>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>沈从文</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>实体书</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>过来亲一下</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>网文作者</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>网文</t>
-        </is>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>这个竹马有点甜</t>
-        </is>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>网文作者</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>网文</t>
-        </is>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
-        <is>
-          <t>道诡异仙</t>
-        </is>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>狐尾的笔</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>网文</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
-        <is>
-          <t>重生八百年后，我被女友抢先表白</t>
-        </is>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>网文作者</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>网文</t>
-        </is>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>重生：学霸和软萌校花的完美人生</t>
-        </is>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>网文作者</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>网文</t>
-        </is>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
-        <is>
-          <t>雪国</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>川端康成</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>实体书</t>
-        </is>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
-        <is>
-          <t>震惊！女帝是我老婆！</t>
-        </is>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>网文作者</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>网文</t>
-        </is>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
-        <is>
-          <t>霍乱时期的爱情</t>
-        </is>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>加西亚·马尔克斯</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>实体书</t>
-        </is>
-      </c>
-    </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
-        <is>
-          <t>飘</t>
-        </is>
-      </c>
-      <c r="B92" t="inlineStr">
-        <is>
-          <t>玛格丽特·米切尔</t>
-        </is>
-      </c>
-      <c r="C92" t="inlineStr">
-        <is>
-          <t>实体书</t>
-        </is>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>骆驼祥子</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>老舍</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>实体书</t>
-        </is>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>高糖倒追：重生女友又凶又萌</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>网文作者</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>网文</t>
         </is>
       </c>
     </row>

</xml_diff>